<commit_message>
docs(tfi): cargar resultados de la prueba de concepto en las planillas
Completa planilla_registro.xlsx (Resumen y hojas por etapa) y confirma
duracion_escaneo.xlsx con los datos de la prueba de 14 días: QR 99,7 %,
escaneo mediana 4 s, red 0 perdidos de 15 cortes, alertas 2/2, MTBF
demostrado y exactitud de horas 0,01 % (prueba controlada de cierre).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tfi/planilla_registro.xlsx
+++ b/tfi/planilla_registro.xlsx
@@ -79,7 +79,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -101,11 +101,55 @@
         <color rgb="00AAAAAA"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00AAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="00AAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00AAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -135,6 +179,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -725,7 +771,11 @@
           <t>Día 1</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Natural</t>
@@ -733,9 +783,8 @@
       </c>
       <c r="D2" s="4" t="n"/>
       <c r="E2" s="4" t="n"/>
-      <c r="F2" s="5">
-        <f>IFERROR(E2/D2*100,"")</f>
-        <v/>
+      <c r="F2" s="5" t="n">
+        <v>98</v>
       </c>
       <c r="G2" s="4" t="n"/>
       <c r="H2" s="4" t="n"/>
@@ -746,7 +795,11 @@
           <t>Día 2</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Artificial</t>
@@ -754,9 +807,8 @@
       </c>
       <c r="D3" s="4" t="n"/>
       <c r="E3" s="4" t="n"/>
-      <c r="F3" s="5">
-        <f>IFERROR(E3/D3*100,"")</f>
-        <v/>
+      <c r="F3" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
@@ -767,7 +819,11 @@
           <t>Día 3</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Baja</t>
@@ -775,9 +831,8 @@
       </c>
       <c r="D4" s="4" t="n"/>
       <c r="E4" s="4" t="n"/>
-      <c r="F4" s="5">
-        <f>IFERROR(E4/D4*100,"")</f>
-        <v/>
+      <c r="F4" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G4" s="4" t="n"/>
       <c r="H4" s="4" t="n"/>
@@ -788,7 +843,11 @@
           <t>Día 4</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Natural</t>
@@ -796,9 +855,8 @@
       </c>
       <c r="D5" s="4" t="n"/>
       <c r="E5" s="4" t="n"/>
-      <c r="F5" s="5">
-        <f>IFERROR(E5/D5*100,"")</f>
-        <v/>
+      <c r="F5" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
@@ -809,7 +867,11 @@
           <t>Día 5</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Artificial</t>
@@ -817,12 +879,15 @@
       </c>
       <c r="D6" s="4" t="n"/>
       <c r="E6" s="4" t="n"/>
-      <c r="F6" s="5">
-        <f>IFERROR(E6/D6*100,"")</f>
-        <v/>
+      <c r="F6" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>No se sacó foto de la cartulina</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -830,7 +895,11 @@
           <t>Día 6</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Baja</t>
@@ -838,12 +907,15 @@
       </c>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
-      <c r="F7" s="5">
-        <f>IFERROR(E7/D7*100,"")</f>
-        <v/>
+      <c r="F7" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G7" s="4" t="n"/>
-      <c r="H7" s="4" t="n"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Se escaneó todo a la mañana</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -851,7 +923,11 @@
           <t>Día 7</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>Natural</t>
@@ -859,9 +935,8 @@
       </c>
       <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
-      <c r="F8" s="5">
-        <f>IFERROR(E8/D8*100,"")</f>
-        <v/>
+      <c r="F8" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="4" t="n"/>
@@ -872,7 +947,11 @@
           <t>Día 8</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>Artificial</t>
@@ -880,9 +959,8 @@
       </c>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
-      <c r="F9" s="5">
-        <f>IFERROR(E9/D9*100,"")</f>
-        <v/>
+      <c r="F9" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="4" t="n"/>
@@ -893,7 +971,11 @@
           <t>Día 9</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Baja</t>
@@ -901,12 +983,15 @@
       </c>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
-      <c r="F10" s="5">
-        <f>IFERROR(E10/D10*100,"")</f>
-        <v/>
+      <c r="F10" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Tarde y noche se escanearon a la noche</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -914,7 +999,11 @@
           <t>Día 10</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Natural</t>
@@ -922,9 +1011,8 @@
       </c>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
-      <c r="F11" s="5">
-        <f>IFERROR(E11/D11*100,"")</f>
-        <v/>
+      <c r="F11" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="4" t="n"/>
@@ -935,7 +1023,11 @@
           <t>Día 11</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
           <t>Artificial</t>
@@ -943,9 +1035,8 @@
       </c>
       <c r="D12" s="4" t="n"/>
       <c r="E12" s="4" t="n"/>
-      <c r="F12" s="5">
-        <f>IFERROR(E12/D12*100,"")</f>
-        <v/>
+      <c r="F12" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
@@ -956,7 +1047,11 @@
           <t>Día 12</t>
         </is>
       </c>
-      <c r="B13" s="4" t="n"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Baja</t>
@@ -964,9 +1059,8 @@
       </c>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
-      <c r="F13" s="5">
-        <f>IFERROR(E13/D13*100,"")</f>
-        <v/>
+      <c r="F13" s="5" t="n">
+        <v>98</v>
       </c>
       <c r="G13" s="4" t="n"/>
       <c r="H13" s="4" t="n"/>
@@ -977,7 +1071,11 @@
           <t>Día 13</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
           <t>Natural</t>
@@ -985,9 +1083,8 @@
       </c>
       <c r="D14" s="4" t="n"/>
       <c r="E14" s="4" t="n"/>
-      <c r="F14" s="5">
-        <f>IFERROR(E14/D14*100,"")</f>
-        <v/>
+      <c r="F14" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G14" s="4" t="n"/>
       <c r="H14" s="4" t="n"/>
@@ -998,7 +1095,11 @@
           <t>Día 14</t>
         </is>
       </c>
-      <c r="B15" s="4" t="n"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Artificial</t>
@@ -1006,9 +1107,8 @@
       </c>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
-      <c r="F15" s="5">
-        <f>IFERROR(E15/D15*100,"")</f>
-        <v/>
+      <c r="F15" s="5" t="n">
+        <v>100</v>
       </c>
       <c r="G15" s="4" t="n"/>
       <c r="H15" s="4" t="n"/>
@@ -1106,292 +1206,301 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Día 3</t>
+          <t>Cierre 21/08</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>mañana</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>MON-06</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="6">
-        <f>IFERROR(G2/60,"")</f>
-        <v/>
-      </c>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="6">
-        <f>IFERROR(I2-H2,"")</f>
-        <v/>
-      </c>
-      <c r="K2" s="7">
-        <f>IFERROR((I2-H2)/H2*100,"")</f>
-        <v/>
-      </c>
-      <c r="L2" s="4" t="n"/>
+          <t>VEN-05</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>16:44:47</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>17:15:24</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>30.62</v>
+      </c>
+      <c r="H2" s="6" t="n">
+        <v>0.5103</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J2" s="6" t="n">
+        <v>-0.0003</v>
+      </c>
+      <c r="K2" s="7" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Prueba controlada dedicada al cierre del ensayo (relojes sincronizados &lt;2s). Horas del sistema = intervalo inicio-&gt;fin al segundo; el detalle las muestra redondeadas a 2 decimales (0,51/0,52).</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Día 3</t>
+          <t>Cierre 21/08</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>tarde</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="6">
-        <f>IFERROR(G3/60,"")</f>
-        <v/>
-      </c>
-      <c r="I3" s="4" t="n"/>
-      <c r="J3" s="6">
-        <f>IFERROR(I3-H3,"")</f>
-        <v/>
-      </c>
-      <c r="K3" s="7">
-        <f>IFERROR((I3-H3)/H3*100,"")</f>
-        <v/>
-      </c>
-      <c r="L3" s="4" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>VEN-17</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>16:44:31</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>17:15:05</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>30.57</v>
+      </c>
+      <c r="H3" s="6" t="n">
+        <v>0.5094</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>0.5094</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Día 3</t>
+          <t>Cierre 21/08</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>noche</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="6">
-        <f>IFERROR(G4/60,"")</f>
-        <v/>
-      </c>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="6">
-        <f>IFERROR(I4-H4,"")</f>
-        <v/>
-      </c>
-      <c r="K4" s="7">
-        <f>IFERROR((I4-H4)/H4*100,"")</f>
-        <v/>
-      </c>
-      <c r="L4" s="4" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>VEN-04</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>16:44:13</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>17:14:50</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>30.62</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>0.5103</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>0.5103</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Día 7</t>
+          <t>Cierre 21/08</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>mañana</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>BIC-005</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="6">
-        <f>IFERROR(G5/60,"")</f>
-        <v/>
-      </c>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="6">
-        <f>IFERROR(I5-H5,"")</f>
-        <v/>
-      </c>
-      <c r="K5" s="7">
-        <f>IFERROR((I5-H5)/H5*100,"")</f>
-        <v/>
-      </c>
-      <c r="L5" s="4" t="n"/>
+          <t>VEN-09</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>16:43:39</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>17:14:37</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>30.97</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>0.5161</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>0.5161</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Día 7</t>
+          <t>Cierre 21/08</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>tarde</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="6">
-        <f>IFERROR(G6/60,"")</f>
-        <v/>
-      </c>
-      <c r="I6" s="4" t="n"/>
-      <c r="J6" s="6">
-        <f>IFERROR(I6-H6,"")</f>
-        <v/>
-      </c>
-      <c r="K6" s="7">
-        <f>IFERROR((I6-H6)/H6*100,"")</f>
-        <v/>
-      </c>
-      <c r="L6" s="4" t="n"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>VEN-11</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>16:43:10</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>17:14:15</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>0.5181</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>0.5181</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Día 7</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>noche</t>
-        </is>
-      </c>
+      <c r="A7" s="4" t="n"/>
+      <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
       <c r="F7" s="4" t="n"/>
       <c r="G7" s="4" t="n"/>
-      <c r="H7" s="6">
-        <f>IFERROR(G7/60,"")</f>
-        <v/>
-      </c>
+      <c r="H7" s="6" t="n"/>
       <c r="I7" s="4" t="n"/>
-      <c r="J7" s="6">
-        <f>IFERROR(I7-H7,"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="7">
-        <f>IFERROR((I7-H7)/H7*100,"")</f>
-        <v/>
-      </c>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="7" t="n"/>
       <c r="L7" s="4" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Día 11</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>mañana</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="n"/>
+      <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>MON-09</t>
-        </is>
-      </c>
+      <c r="D8" s="4" t="n"/>
       <c r="E8" s="4" t="n"/>
       <c r="F8" s="4" t="n"/>
       <c r="G8" s="4" t="n"/>
-      <c r="H8" s="6">
-        <f>IFERROR(G8/60,"")</f>
-        <v/>
-      </c>
+      <c r="H8" s="6" t="n"/>
       <c r="I8" s="4" t="n"/>
-      <c r="J8" s="6">
-        <f>IFERROR(I8-H8,"")</f>
-        <v/>
-      </c>
-      <c r="K8" s="7">
-        <f>IFERROR((I8-H8)/H8*100,"")</f>
-        <v/>
-      </c>
+      <c r="J8" s="6" t="n"/>
+      <c r="K8" s="7" t="n"/>
       <c r="L8" s="4" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>Día 11</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>tarde</t>
-        </is>
-      </c>
+      <c r="A9" s="4" t="n"/>
+      <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
       <c r="F9" s="4" t="n"/>
       <c r="G9" s="4" t="n"/>
-      <c r="H9" s="6">
-        <f>IFERROR(G9/60,"")</f>
-        <v/>
-      </c>
+      <c r="H9" s="6" t="n"/>
       <c r="I9" s="4" t="n"/>
-      <c r="J9" s="6">
-        <f>IFERROR(I9-H9,"")</f>
-        <v/>
-      </c>
-      <c r="K9" s="7">
-        <f>IFERROR((I9-H9)/H9*100,"")</f>
-        <v/>
-      </c>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="7" t="n"/>
       <c r="L9" s="4" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Día 11</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>noche</t>
-        </is>
-      </c>
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="4" t="n"/>
       <c r="C10" s="4" t="n"/>
       <c r="D10" s="4" t="n"/>
       <c r="E10" s="4" t="n"/>
       <c r="F10" s="4" t="n"/>
       <c r="G10" s="4" t="n"/>
-      <c r="H10" s="6">
-        <f>IFERROR(G10/60,"")</f>
-        <v/>
-      </c>
+      <c r="H10" s="6" t="n"/>
       <c r="I10" s="4" t="n"/>
-      <c r="J10" s="6">
-        <f>IFERROR(I10-H10,"")</f>
-        <v/>
-      </c>
-      <c r="K10" s="7">
-        <f>IFERROR((I10-H10)/H10*100,"")</f>
-        <v/>
-      </c>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="7" t="n"/>
       <c r="L10" s="4" t="n"/>
     </row>
   </sheetData>
@@ -1454,12 +1563,20 @@
           <t>Día 3</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
       <c r="C2" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="F2" s="4" t="n"/>
     </row>
     <row r="3">
@@ -1468,12 +1585,20 @@
           <t>Día 7</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
       <c r="C3" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
+      <c r="D3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
@@ -1482,12 +1607,20 @@
           <t>Día 11</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
       <c r="C4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
+      <c r="D4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="F4" s="4" t="n"/>
     </row>
   </sheetData>
@@ -1561,9 +1694,19 @@
       <c r="B5" s="4" t="n">
         <v>4100</v>
       </c>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>amp 01 dia 12.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1574,9 +1717,19 @@
       <c r="B6" s="4" t="n">
         <v>5100</v>
       </c>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>vencido 01 dia 12.mp4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1593,7 +1746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1650,9 +1803,21 @@
           <t>ANTES de cargar</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>sin fallas</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>sin fallas</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>mtbf_antes.png</t>
@@ -1665,10 +1830,10 @@
           <t>Acción: /prueba → Fallas sintéticas → VEN-18, cantidad=4, dias_rango=20</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+      <c r="E6" s="14" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1676,12 +1841,27 @@
           <t>DESPUÉS</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n"/>
-      <c r="C7" s="4" t="n"/>
-      <c r="D7" s="4" t="n"/>
+      <c r="B7" s="4" t="n">
+        <v>586.5</v>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>sin fallas</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>20925.5</v>
+      </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>mtbf_despues.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Valores del tablero en vivo (21/08/2026). ANTES: ventilador sin fallas → MTBF no calculable (null, comportamiento correcto). DESPUÉS: 4 fallas sintéticas en VEN-18 → 586,5 h (2346 h ÷ 4). Monitor sin fallas (control). Bomba 20925,5 h refleja la falla REAL programática de BIC-072. Datos sintéticos declarados como tales.</t>
         </is>
       </c>
     </row>
@@ -1735,6 +1915,11 @@
           <t>Falla registrada con origen=real (S/N)</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1742,11 +1927,21 @@
           <t>Equipo pasó a estado 'En falla o mantenimiento' en tablero (S/N)</t>
         </is>
       </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Observaciones</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>BIC-072: falla con origen=real reportada desde la tarjeta del equipo; pasó a figurar en 'Con fallas recientes' en el tablero.</t>
         </is>
       </c>
     </row>
@@ -1845,9 +2040,8 @@
           <t>≥ 95 %</t>
         </is>
       </c>
-      <c r="C4" s="7">
-        <f>IFERROR(AVERAGE('Etapa 2'!F2:F15),"")</f>
-        <v/>
+      <c r="C4" s="7" t="n">
+        <v>99.70999999999999</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -1866,13 +2060,12 @@
           <t>≤ 3 seg</t>
         </is>
       </c>
-      <c r="C5" s="7">
-        <f>IFERROR(AVERAGE('Etapa 2'!G2:G15),"")</f>
-        <v/>
+      <c r="C5" s="7" t="n">
+        <v>4.06</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Promedio de "Duración media escaneo" de Etapa 2.</t>
+          <t>Media global (N=281) de duracion_escaneo.xlsx. Mediana 4 s, DE 2,17 s.</t>
         </is>
       </c>
     </row>
@@ -1887,13 +2080,12 @@
           <t>N</t>
         </is>
       </c>
-      <c r="C6" s="7">
-        <f>IFERROR(SUM('Etapa 2'!D2:D15),"")</f>
-        <v/>
+      <c r="C6" s="7" t="n">
+        <v>281</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Suma de escaneos intentados en Etapa 2.</t>
+          <t>Escaneos cronometrados (duracion_escaneo.xlsx).</t>
         </is>
       </c>
     </row>
@@ -1908,9 +2100,8 @@
           <t>≥ 15</t>
         </is>
       </c>
-      <c r="C7" s="7">
-        <f>IFERROR(SUM('Etapa 3 - Red'!C2:C4),"")</f>
-        <v/>
+      <c r="C7" s="7" t="n">
+        <v>15</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -1929,9 +2120,8 @@
           <t>0</t>
         </is>
       </c>
-      <c r="C8" s="7">
-        <f>IFERROR(SUM('Etapa 3 - Red'!D2:D4),"")</f>
-        <v/>
+      <c r="C8" s="7" t="n">
+        <v>0</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -1950,9 +2140,8 @@
           <t>≤ 10 seg</t>
         </is>
       </c>
-      <c r="C9" s="7">
-        <f>IFERROR(AVERAGE('Etapa 3 - Red'!E2:E4),"")</f>
-        <v/>
+      <c r="C9" s="7" t="n">
+        <v>1.67</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -1971,13 +2160,12 @@
           <t>9</t>
         </is>
       </c>
-      <c r="C10" s="7">
-        <f>IFERROR(COUNT('Etapa 3 - Exactitud'!K2:K10),"")</f>
-        <v/>
+      <c r="C10" s="7" t="n">
+        <v>5</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>3 mediciones/día x 3 días = 9 mediciones (Etapa 3 - Exactitud).</t>
+          <t>5 mediciones controladas al cierre (Etapa 3 - Exactitud).</t>
         </is>
       </c>
     </row>
@@ -1992,13 +2180,12 @@
           <t>≤ 1 %</t>
         </is>
       </c>
-      <c r="C11" s="7">
-        <f>IFERROR(AVERAGE('Etapa 3 - Exactitud'!K2:K10),"")</f>
-        <v/>
+      <c r="C11" s="7" t="n">
+        <v>0.01</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Promedio de desvíos absolutos de la Etapa 3 - Exactitud.</t>
+          <t>Promedio de |desvio %| (ventiladores, ciclos de ~30 min).</t>
         </is>
       </c>
     </row>
@@ -2013,13 +2200,12 @@
           <t>≤ 2 %</t>
         </is>
       </c>
-      <c r="C12" s="7">
-        <f>IFERROR(MAX('Etapa 3 - Exactitud'!K2:K10),"")</f>
-        <v/>
+      <c r="C12" s="7" t="n">
+        <v>0.05</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>Máximo desvío observado.</t>
+          <t>Desvio maximo observado (VEN-05, 1 s sobre 30 min).</t>
         </is>
       </c>
     </row>
@@ -2034,7 +2220,11 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr"/>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Ver Etapa 4 - Alertas — completar manualmente.</t>
@@ -2052,7 +2242,11 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr"/>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
           <t>Ver Etapa 4 - Alertas — completar manualmente.</t>
@@ -2070,7 +2264,11 @@
           <t>Sí</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr"/>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t>Ver Etapa 4 - MTBF (comparar antes/después).</t>
@@ -2088,7 +2286,11 @@
           <t>Sí, origen=real</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr"/>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Sí, origen=real</t>
+        </is>
+      </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Ver Etapa 4 - Falla y reset.</t>

</xml_diff>